<commit_message>
Update asset metadata and delivery documentation for Uraba project
Replit-Commit-Author: Agent
</commit_message>
<xml_diff>
--- a/entregables/Mibet_Lista_Verificacion_Uraba_Agrivoltaico.xlsx
+++ b/entregables/Mibet_Lista_Verificacion_Uraba_Agrivoltaico.xlsx
@@ -1492,7 +1492,7 @@
       <c r="G23" s="63" t="n"/>
       <c r="H23" s="73" t="inlineStr">
         <is>
-          <t>2.5 m (agrivoltaico: paso de cultivo/maquinaria bajo los paneles)</t>
+          <t>3.0 m (agrivoltaico: borde inferior del panel a 3 m del suelo — cultivo y maquinaria debajo)</t>
         </is>
       </c>
       <c r="I23" s="63" t="n"/>
@@ -1568,7 +1568,7 @@
       <c r="B27" s="7" t="n"/>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>Agrivoltaico: 3.200 m² de terreno, ocupación FV 30% (960 m²). Estructura elevada 2.5 m con corredores entre matrices para cultivo. Plano de disposición se enviará junto con el informe de suelo.</t>
+          <t>Agrivoltaico: 3.200 m² de terreno (32 × 100 m), ocupación FV 30% (960 m²). Estructura elevada 3.0 m con corredores de cultivo de ~4 m entre filas. Se adjunta plano de disposición; informe de suelo pendiente.</t>
         </is>
       </c>
       <c r="D27" s="7" t="n"/>

</xml_diff>